<commit_message>
Mise à jour IG 5bf0f7cc188d4fc058dd0713b4d3765be79c7fa0
</commit_message>
<xml_diff>
--- a/structureIG/ig/StructureDefinition-fr-composition-document-ips.xlsx
+++ b/structureIG/ig/StructureDefinition-fr-composition-document-ips.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-18T13:56:24+00:00</t>
+    <t>2026-09-21T13:38:34+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -3959,10 +3959,10 @@
     <t>Composition.section:sectionPlanOfCare.entry</t>
   </si>
   <si>
-    <t>Composition.section:sectionPlanOfCare.entry:demandeDexamenOuDeSuivi</t>
-  </si>
-  <si>
-    <t>demandeDexamenOuDeSuivi</t>
+    <t>Composition.section:sectionPlanOfCare.entry:serviceRequest</t>
+  </si>
+  <si>
+    <t>serviceRequest</t>
   </si>
   <si>
     <t xml:space="preserve">Reference(https://interop.esante.gouv.fr/ig/fhir/document-core/StructureDefinition/fr-service-request-document|0.1.0)
@@ -3972,10 +3972,10 @@
     <t>Entrée Demande d examen ou de suivi</t>
   </si>
   <si>
-    <t>Composition.section:sectionPlanOfCare.entry:traitement</t>
-  </si>
-  <si>
-    <t>traitement</t>
+    <t>Composition.section:sectionPlanOfCare.entry:medicationRequest</t>
+  </si>
+  <si>
+    <t>medicationRequest</t>
   </si>
   <si>
     <t xml:space="preserve">Reference(https://interop.esante.gouv.fr/ig/fhir/document-core/StructureDefinition/fr-medication-request-document|0.1.0)
@@ -3985,10 +3985,10 @@
     <t>Entrée Traitement</t>
   </si>
   <si>
-    <t>Composition.section:sectionPlanOfCare.entry:vaccinRecommande</t>
-  </si>
-  <si>
-    <t>vaccinRecommande</t>
+    <t>Composition.section:sectionPlanOfCare.entry:immunizationRecommendation</t>
+  </si>
+  <si>
+    <t>immunizationRecommendation</t>
   </si>
   <si>
     <t xml:space="preserve">Reference(https://interop.esante.gouv.fr/ig/fhir/document-core/StructureDefinition/fr-immunization-recommendation-document|0.1.0)

</xml_diff>